<commit_message>
Log first PIWA prospecting emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9KJnaVmdH42r75H4m1WYx
</commit_message>
<xml_diff>
--- a/prospection/prospects-PIWA-500.xlsx
+++ b/prospection/prospects-PIWA-500.xlsx
@@ -7,13 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retirés" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal envois" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lot 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retirés" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Prospects'!$A$1:$R$524</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Prospects'!$A$1:$R$524</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -86,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -113,6 +114,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,6 +480,371 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="n"/>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Adresse</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Objet</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Depuis</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Résultat</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Relance prévue le</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Studio218</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>contact@studio218.fr</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ajouter la vidéo à vos offres web, sans recruter</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>YouLoveWords</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>contact@youlovewords.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Transformer vos contenus écrits en vidéos</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Conceptory</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>info@conceptory.fr</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Un renfort motion design pour vos formats sociaux</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Gust</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>contact@agencegust.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Absorber vos pics de production vidéo, en 25 langues</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Hula Hoop</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>contact@hula-hoop.fr</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Des vidéos multilingues pour vos clients internationaux</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Adveris</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>contact@adveris.fr</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Des vidéos courtes pour vos campagnes social ads</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Madaré</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>contact@madare.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>La vidéo pour prolonger vos projets de marque</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Hi Agency</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>contact@hi-agency.fr</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Un renfort vidéo pour vos marques, en France et en Suisse</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -579,7 +946,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -625,10 +992,14 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="260" customHeight="1">
@@ -671,11 +1042,15 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>Non envoyé</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
-      <c r="I4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Écarté : semble être un lieu de séminaires, pas une agence</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="260" customHeight="1">
       <c r="A5" s="3" t="n">
@@ -717,10 +1092,14 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="260" customHeight="1">
@@ -763,7 +1142,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -809,7 +1188,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
@@ -855,7 +1234,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -901,7 +1280,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -947,7 +1326,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -993,7 +1372,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -1039,7 +1418,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -1085,7 +1464,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -1131,7 +1510,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -1177,7 +1556,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1223,7 +1602,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -1269,7 +1648,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1315,7 +1694,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -1361,7 +1740,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1407,7 +1786,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Prêt, non envoyé</t>
+          <t>En attente : adresse mail introuvable</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -1418,7 +1797,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1708,10 +2087,14 @@
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q3" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="110" customHeight="1">
@@ -1796,10 +2179,14 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="110" customHeight="1">
@@ -1884,10 +2271,14 @@
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q5" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="110" customHeight="1">
@@ -2060,10 +2451,14 @@
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q7" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="110" customHeight="1">
@@ -2148,10 +2543,14 @@
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q8" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="110" customHeight="1">
@@ -2324,10 +2723,14 @@
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q10" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R10" s="3" t="inlineStr"/>
     </row>
     <row r="11" ht="110" customHeight="1">
@@ -2412,10 +2815,14 @@
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q11" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R11" s="3" t="inlineStr"/>
     </row>
     <row r="12" ht="110" customHeight="1">
@@ -2676,10 +3083,14 @@
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="110" customHeight="1">
@@ -49050,7 +49461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -49187,7 +49598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Log Gravotech and Vates emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9KJnaVmdH42r75H4m1WYx
</commit_message>
<xml_diff>
--- a/prospection/prospects-PIWA-500.xlsx
+++ b/prospection/prospects-PIWA-500.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -829,6 +829,80 @@
         </is>
       </c>
       <c r="G10" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Gravotech</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>contact@gravotech.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Préparer Global Industrie 2027 en vidéo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Envoyé (adresse publiée dans leurs mentions légales)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Vates</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>sales@vates.tech</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Une vidéo pour présenter Vates après votre levée de 30 M€</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Envoyé (adresse publiée sur leur site d'aide)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>
@@ -3703,10 +3777,14 @@
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q21" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R21" s="3" t="inlineStr"/>
     </row>
     <row r="22" ht="110" customHeight="1">
@@ -5314,10 +5392,14 @@
       </c>
       <c r="P39" s="3" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="Q39" s="3" t="inlineStr"/>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="Q39" s="3" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
       <c r="R39" s="3" t="inlineStr"/>
     </row>
     <row r="40" ht="110" customHeight="1">

</xml_diff>

<commit_message>
Log second wave of PIWA prospecting emails
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9KJnaVmdH42r75H4m1WYx
</commit_message>
<xml_diff>
--- a/prospection/prospects-PIWA-500.xlsx
+++ b/prospection/prospects-PIWA-500.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,956 @@
         </is>
       </c>
       <c r="G12" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pickers</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>contact@agence-pickers.fr</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Espaces Atypiques</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>contact@espaces-atypiques.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vulcania</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>bienvenue@vulcania.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Fermob</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>info@fermob.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Festival des Vieilles Charrues</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>info@vieillescharrues.asso.fr</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Office de Tourisme du Lac d'Annecy</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>info@lac-annecy.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Aura Aero</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>contact@aura-aero.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Quobly</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>contact@quobly.io</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>GitGuardian</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>contact@gitguardian.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kipli</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>hello@kipli.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Groupe Giboire</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>communication@giboire.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gobelins Paris</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>info-il@gobelins.fr</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ÉCHEC : bloqué par le serveur du destinataire</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Voltalia</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>contact@voltalia.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ÉCHEC : bloqué par le serveur du destinataire</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Maisons du Monde</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>presse@maisonsdumonde.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Puy du Fou</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>servicepresse@puydufou.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Groupe Barrière</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>contact-presse@groupebarriere.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Groupe Rocher</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>press@yr.net</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ÉCHEC : adresse inexistante</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Rubis</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>presse@rubis.fr</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Latécoère</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>latecoeregroupcommunication@latecoere.aero</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Asmodee</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>press@asmodee.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Mecachrome</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>communication@mecachromegroup.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Lectra</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>presse@lectra.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Trigano</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>communication@trigano.fr</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Figeac Aéro</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>communications.group@figeac-aero.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Lacroix Group</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>info@lacroix-group.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Groupe Guillin</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>contact@groupeguillin.fr</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>(personnalisé)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>

</xml_diff>

<commit_message>
Log third wave of PIWA emails and price follow-ups
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9KJnaVmdH42r75H4m1WYx
</commit_message>
<xml_diff>
--- a/prospection/prospects-PIWA-500.xlsx
+++ b/prospection/prospects-PIWA-500.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1850,6 +1850,853 @@
         </is>
       </c>
       <c r="G38" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>(33 sociétés déjà contactées)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>réponse dans chaque conversation</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Complément : tous les tarifs dès 390 € HT + exemples sur demande</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Envoyé</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Laforêt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>contact-laforet@laforet.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Des vidéos pour tout le réseau Laforêt, dès 390 € HT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Keep Cool</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>contact@keepcool.fr</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Des vidéos pour tout le réseau Keep Cool, dès 390 € HT</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>presse@ada.fr</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Des vidéos pour tout le réseau ADA, dès 390 € HT</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Elsan</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>news@elsan.care</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Elsan, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Groupe BPCE</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>presse@bpce.fr</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Une vidéo pour le Groupe BPCE, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Groupe RATP</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>servicedepresse@ratp.fr</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Une vidéo pour le Groupe RATP, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bouygues</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>presse@bouygues.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Bouygues, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Pichet</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>contact@pichet.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Pichet, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Niryo</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>contact@niryo.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Niryo, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Technature</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>info@tech-nature.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Technature, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Enedis</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>service-presse@enedis.fr</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Enedis, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Mutuelle de Poitiers Assurances</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>accueil@mutuelledepoitiers.fr</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Mutuelle de Poitiers Assurances, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Seb</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>presse@groupeseb.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Une vidéo pour le Groupe SEB, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>DomusVi</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>press@domusvi.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Une vidéo pour DomusVi, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>OVHcloud</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>media@ovhcloud.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Une vidéo pour OVHcloud, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Teleperformance</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>tppublicaffairs@teleperformance.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Teleperformance, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Getlink</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>press@getlinkgroup.com</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Getlink, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>bioMérieux</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>media@biomerieux.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Une vidéo pour bioMérieux, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Servier</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>presse@servier.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Servier, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Air Liquide</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>media@airliquide.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Air Liquide, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Alstom</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>mediarelations@alstomgroup.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Une vidéo pour Alstom, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Groupe Beneteau</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>presse@beneteau-group.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Une vidéo pour le Groupe Beneteau, dès 390 € HT, livrée en 7 jours</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>piwastudiopiwastudio@gmail.com</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Envoyé, pas de retour en erreur</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
         <is>
           <t>12/10/2026</t>
         </is>

</xml_diff>